<commit_message>
Add standardized_caafimaad_master.xlsx dataset to raw_dataset directory
</commit_message>
<xml_diff>
--- a/laacibnet_curated_dataset.xlsx
+++ b/laacibnet_curated_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D627"/>
+  <dimension ref="A1:D673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14210,6 +14210,1018 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>FA-ga Ingiriiska Oo Ganaax Culus Dul Dhigay Mid Kamid Ah Weeraryahannada Chelsea</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/fa-ga-ingiriiska-oo-ganaax-culus-dul-dhigay-mid-kamid-ah-weeraryahannada-chelsea/</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Neymar Oo Shaaciyay Labada Xul Ee Uu Doonayo Inay Isugu Yimaadaan Final-ka Koobka Adduunka</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/neymar-oo-shaaciyay-labada-dal-ee-uu-doonayo-inay-isugu-yimaadaan-final-ka-koobka-adduunka/</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Thierry Henry Oo Kashifay Sirta Guulaha Arsenal Ee Xilli Ciyaareed Kaan Ka Hor Kulanka Atletico Madrid</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/thierry-henry-oo-kashifay-sirta-guulaha-arsenal-ee-xilli-ciyaareed-kaan-ka-hor-kulanka-atletico-madrid/</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>PSG Mise Bayern? – Wayne Rooney Oo Shaaciyay Kooxda Uu Aaminsan Yahay Inay U Soo Gudbeyso Final-ka Tartanka Champions League-ga</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/psg-mise-bayern-wayne-rooney-oo-shaaciyay-kooxda-uu-aaminsan-yahay-inay-u-soo-gudbeyso-final-ka-tartanka-champions-league-ga/</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Odegaard Oo Shaaca Ka Qaaday Xiddiga Ka Dhiga Arsenal Mid Halis Badan Oo Ay Kooxaha Ka Argagaxaan</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/odegaard-oo-shaaca-ka-qaaday-xiddiga-ka-dhiga-arsenal-mid-halis-badan-oo-ay-kooxaha-ka-argagaxaan/</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Obi Mikel Oo Shaaciyay Xiddig Chelsea Ah Oo Ku Faa’iday Ceydhintii Liam Rosenior</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/obi-mikel-oo-shaaciyay-xiddig-chelsea-ah-oo-ku-faaiday-ceydhintii-liam-rosenior/</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>WARBIXIN: Qorshaha Liverpool Ee Suuqa Xagaaga</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/warbixin-qorshaha-liverpool-ee-suuqa-xagaaga/</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Shaxda Ay Arsenal Kaga Hor Tagi Karto Atletico Kulanka Caawa</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/shaxda-ay-arsenal-kaga-hor-tagi-karto-atletico-kulanka-caawa/</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Labada Tababare Ee Ugu Cad-cad Shaqada Real Madrid Oo La Shaaciyay</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/labada-tababare-ee-ugu-cad-cad-shaqada-real-madrid-oo-la-shaaciyay/</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Mikel Arteta Oo Shaaca Ka Qaaday Qorshaha Ay Kooxdiisa Ku Wajaheyso Atletico Kulanka Caawa</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/mikel-arteta-oo-shaaca-ka-qaaday-qorshaha-ay-kooxdiisa-ku-wajaheyso-atletico-kulanka-caawa/</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Malouda Oo Chelsea Ugu Baaqay Saxiixa Weeraryahan Ay City Heshiis Hordhac Ah La Gaartay</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/malouda-oo-chelsea-ugu-baaqay-saxiixa-weeraryahan-ay-city-heshiis-hordhac-ah-la-gaartay/</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Obi Mikel Oo Shaaciyay Tababaraha Loo Baahan Yahay In Chelsea Ay Magacowdo Kadib Ceydhintii Liam Rosenior</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/obi-mikel-oo-shaaciyay-tababaraha-loo-baahan-yahay-in-chelsea-ay-magacowdo-kadib-ceydhintii-liam-rosenior/</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Thierry Henry Oo Arsenal Uga Digay Awoodda Atletico Ka Hor Kulanka Semi-final-ka Ee Champions League-ga</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/thierry-henry-oo-arsenal-uga-digay-awoodda-atletico-ka-hor-kulanka-semi-final-ka-ee-champions-league-ga/</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Rooney Oo Dhaleeceeyay Tababaraha PSG, Shaaciyayna Meesha Kaliya Ay Ka Liidato Bayern</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/rooney-oo-dhaleeceeyay-tababaraha-psg-shaaciyayna-meesha-kaliya-ay-ka-liidato-bayern/</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Martin Odegaard Oo Go’aan Culus Ka Soo Saaray Mustaqbalkiisa Arsenal</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/martin-odegaard-oo-goaan-culus-ka-soo-saaray-mustaqbalkiisa-arsenal/</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Joe Cole Oo Daaha Ka Rogay Hal Arrin Oo Palmer Ku Qasbi Karta Inuu Chelsea Ka Tago</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/joe-cole-oo-daaha-ka-rogay-hal-arrin-oo-palmer-ku-qasbi-karta-inuu-chelsea-ka-tago/</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Clarence Seedorf Oo Magacaabay Kooxda Ugu Cadcad Ku Guuleysiga Champions League Sannad Kaan; Ma Ahan PSG</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/clarence-seedorf-oo-magacaabay-kooxda-ugu-cadcad-ku-guuleysiga-champions-league-sannad-kaan-ma-ahan-psg/</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Luis Enrique Oo Shaaciyay Kulankii Ugu Adkaa Ee Uu Koox Leyliyo, Iyo Goolasha Ay Kooxdiisu Dhalin Doonto Ciyaarta Lugta Labaad Ee Munich</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/luis-enrique-oo-shaaciyay-kulankii-ugu-adkaa-ee-uu-koox-leyliyo-iyo-goolasha-ay-kooxdiisu-dhalin-doonto-ciyaarta-lugta-labaad-ee-munich/</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Mikel Arteta Oo Xaqiijiyay Xiddigihiisa Diyaarka U Ah Kulanka Atletico Iyo Kuwa Seegaya</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/mikel-arteta-oo-xaqiijiyay-xiddigihiisa-diyaarka-u-ah-kulanka-atletico-iyo-kuwa-seegaya/</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Rio Ferdinand Oo Magacaabay Xiddiga Ku Hoggaamin Kara Arsenal Ku Guuleysiga Horyaalka Xilli Ciyaareed Kaan</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/rio-ferdinand-oo-magacaabay-xiddiga-ku-hoggaamin-kara-arsenal-ku-guuleysiga-horyaalka-xilli-ciyaareed-kaan/</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Casemiro Oo Iska Diiday Dalab Weyn Oo Uga Yimid Sacuudiga, Oggolaadayna Inuu Ku Biiro Koox Ka Dhisan Horyaalka Mareykanka</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/casemiro-oo-iska-diiday-dalab-weyn-oo-uga-yimid-sacuudiga-oggolaadayna-inuu-ku-biiro-koox-ka-dhisan-horyaalka-mareykanka/</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Florentino Pérez Oo Doortay Tababaraha Beddelaya Alvaro Arbeloa</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/florentino-perez-oo-doortay-tababaraha-beddelaya-alvaro-arbeloa/</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Manuel Ugarte Oo Go’aan Ka Gaartay Mustaqbalka Manuel Ugarte</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/manuel-ugarte-oo-goaan-ka-gaartay-mustaqbalka-manuel-ugarte/</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Sergio Aguero Oo Magacaabay Kooxda Ugu Cadcad Ku Guuleysiga Champions League Ka Hor Kulamada Semi-final-ka Tartanka</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/sergio-aguero-oo-magacaabay-kooxda-ugu-cadcad-ku-guuleysiga-champions-league-ka-hor-kulamada-semi-final-ka-tartanka/</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Arsenal Oo War Farxad Leh Ka Heshay Xaaladda Eze iyo Calafiori Ka Hor Kulanka Atletico</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/arsenal-oo-war-farxad-leh-ka-heshay-xaaladda-eze-iyo-calafiori-ka-hor-kulanka-lugta-atletico/</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Guti Oo Real Madrid Kaga Digay Inay Tababareheeda Cusub U Magacowdo Mourinho; Sabab?</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/guti-oo-real-madrid-kaga-digay-inay-tababareheeda-cusub-u-magacowdo-mourinho-sabab/</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Sesko: “Aad Ayaan Uga Soo Hor Jeedaa Inuu Isaga Innaga Tago”</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/sesko-aad-ayaan-uga-soo-hor-jeedaa-inuu-isaga-innaga-tago/</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Paul Pogba Iyo Jesse Lingard Oo Si Wadajir Ah U Tilmaamay Xiddig United U Ciyaara Oo Mudan Abaalmarinta Ballon d’Or Ee Sannad Kaan</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/paul-pogba-iyo-jesse-lingard-oo-si-wadajir-ah-u-tilmaamay-xiddig-united-u-ciyaara-oo-mudan-abaalmarinta-ballon-dor-ee-sannad-kaan/</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Obi Mikel Oo Shaaciyay Cidda Chelsea Ka Saari Karta Xaaladda Xun Ay Ku Sugan Tahay Waqti Xaadir Kaan</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/obi-mikel-oo-shaaciyay-cidda-chelsea-ka-saari-karta-xaaladda-xun-ay-ku-sugan-tahay-waqti-xaadir-kaan/</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Maguire Oo Weerar Afka Ah Kabaha Kula Dul-maray Ruben Amorim</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/maguire-oo-weerar-afka-ah-kabaha-kula-dul-maray-ruben-amorim/</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>WAR WEYN! Julián Álvarez Oo Oggolaaday Inuu Ku Biiro Barcelona</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/war-weyn-julian-alvarez-oo-oggolaaday-inuu-ku-biiro-barcelona/</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Gary Neville Oo Shaaciyay Kulanka Go’aaminaya Mustaqbalka Arne Slot Ee Liverpool</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/gary-neville-oo-shaaciyay-kulanka-goaaminaya-mustaqbalka-arne-slot-ee-liverpool/</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Gerrard Oo Farta Ku Fiiqay Xiddiga Uu U Arko Kan Ugu Muhiimsan Chelsea Xilli Ciyaareed Kaan</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/gerrard-oo-farta-ku-fiiqay-xiddiga-uu-u-arko-kan-ugu-muhiimsan-chelsea-xilli-ciyaareed-kaan/</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Supercomputer-ka Opta Oo Saadaaliyay 5-ta Koox Ee Premier League Ee Usoo Bixi Doona Champions League Xilli Ciyaareedka Dambe</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/supercomputer-ka-opta-oo-saadaaliyay-5-ta-koox-ee-premier-league-ee-usoo-bixi-doona-champions-league-xilli-ciyaareedka-dambe/</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Taageerayaasha Manchester United Oo Codsi Lama Filaan Ah U Diray Casemiro Kadib Kulankii Brentford</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/taageerayaasha-manchester-united-oo-codsi-lama-filaan-ah-u-diray-casemiro-kadib-kulankii-brentford/</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Bruno Fernandes Oo Barbareeyay Rikoodh Muhiim Ah Oo Uu Dhigay Cristiano Ronaldo</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/bruno-fernandes-oo-barbareeyay-rikoodh-muhiim-ah-oo-uu-dhigay-cristiano-ronaldo/</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Supercomputer-ka Opta Oo Saadaaliyay Kooxda Ugu Cad-cad Ku Guuleysiga Champions League Ka Hor Kulamada Semi-final-ka</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/supercomputer-ka-opta-oo-saadaaliyay-kooxda-ugu-cad-cad-ku-guuleysiga-champions-league-ka-hor-kulamada-semi-final-ka/</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Jamie Carragher Oo Shaaciyay Caqabadda Ugu Weyn Ee Arsenal Ka Hor Istaagi Karta Ku Guuleysiga Horyaalka Xilli Ciyaareed Kaan</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/jamie-carragher-oo-shaaciyay-caqabadda-ugu-weyn-ee-arsenal-ka-hor-istaagi-karta-ku-guuleysiga-horyaalka-xilli-ciyaareed-kaan/</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Michael Carrick Oo Amaan Ugu Qubeeyay Mainoo Kadib Guushii Brentford</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/michael-carrick-oo-amaan-ugu-qubeeyay-mainoo-kadib-guushii-brentford/</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Gary Lineker Oo Shaaciyay Kulanka Kaliya Ee Arsenal Ka Hor Istaagi Kara Ku Guuleysiga Horyaalka Xilli Ciyaareed Kaan</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/gary-lineker-oo-shaaciyay-kulanka-kaliya-ee-arsenal-ka-hor-istaagi-kara-ku-guuleysiga-horyaalka-xilli-ciyaareed-kaan/</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Paul Merson Oo Magacaabay Tababaraha Ay Tahay In Loo Dhiibo Shaqada Chelsea Xilli Ciyaareedka Dambe</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/paul-merson-oo-magacaabay-tababaraha-ay-tahay-inuu-qabto-shaqada-chelsea-xilli-ciyaareedka-dambe/</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Jamie Carragher Oo Farta Ku Fiiqay Cidda Uu Aaminsan Yahay Inay Noqoneyso Tababaraha Joogtada Ah Ee Manchester United Xilli Ciyaareedka Dambe</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/jamie-carragher-oo-shaaciyay-cidda-noqoneysa-tababaraha-joogtada-ah-ee-manchester-united-xilli-ciyaareedka-dambe/</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Chelsea Oo Ku Dhawaaqday Waqtiga Ay Magacaabeyso Tababare Rasmi Ah</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/chelsea-oo-ku-dhawaaqday-waqtiga-ay-magacaabeyso-tababare-rasmi-ah/</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Muxuu Carrick Ka Yiri Guushii Kooxdiisa Ay Ka Gaartay Brentford?</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/muxuu-carrick-ka-yiri-guushii-kooxdiisa-ay-ka-gaartay-brentford/</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Manchester United Oo Guul Muhiim Ah Ka Gaartay Brentford</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/manchester-united-oo-guul-muhiim-ah-ka-gaartay-brentford/</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Bruno Fernandes Oo Qarka U Saaran Inuu Jebiyo Rikoodh Uu Ku Faano Kevin De Bruyne</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>https://www.laacibnet.net/bruno-fernandes-oo-qarka-u-saaran-inuu-jebiyo-rikoodh-uu-ku-faano-kevin-de-bruyne/</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>ciyaaraha_maanta</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>laacibnet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>